<commit_message>
refactor: switch numerical demo to Genshin-like theme (sanitized)
- weapons: 单手剑/双手剑/长柄武器/弓/法器 instead of Honkai paths
- elements: 火水雷冰风岩
- skills: 普通攻击/元素战技/元素爆发
- items: 摩拉/原石/相遇之缘/命星
- enemies: 遗迹机兵/风蚀之核
- fictional character names (炎锋·旅者 etc.)
- regenerate demo configs + HTML report
</commit_message>
<xml_diff>
--- a/demo/configs/EnemyConfig.xlsx
+++ b/demo/configs/EnemyConfig.xlsx
@@ -43,7 +43,7 @@
     <t>2001</t>
   </si>
   <si>
-    <t>裂界造物·Lv5</t>
+    <t>遗迹机兵·Lv5</t>
   </si>
   <si>
     <t>5</t>
@@ -67,7 +67,7 @@
     <t>2002</t>
   </si>
   <si>
-    <t>裂界造物·Lv10</t>
+    <t>遗迹机兵·Lv10</t>
   </si>
   <si>
     <t>10</t>
@@ -85,7 +85,7 @@
     <t>2003</t>
   </si>
   <si>
-    <t>裂界造物·Lv15</t>
+    <t>遗迹机兵·Lv15</t>
   </si>
   <si>
     <t>15</t>
@@ -103,7 +103,7 @@
     <t>2004</t>
   </si>
   <si>
-    <t>裂界造物·Lv20</t>
+    <t>遗迹机兵·Lv20</t>
   </si>
   <si>
     <t>20</t>
@@ -121,7 +121,7 @@
     <t>2005</t>
   </si>
   <si>
-    <t>裂界造物·Lv25</t>
+    <t>遗迹机兵·Lv25</t>
   </si>
   <si>
     <t>25</t>
@@ -139,7 +139,7 @@
     <t>2006</t>
   </si>
   <si>
-    <t>裂界造物·Lv30</t>
+    <t>遗迹机兵·Lv30</t>
   </si>
   <si>
     <t>30</t>
@@ -157,7 +157,7 @@
     <t>2007</t>
   </si>
   <si>
-    <t>裂界造物·Lv35</t>
+    <t>遗迹机兵·Lv35</t>
   </si>
   <si>
     <t>35</t>
@@ -175,7 +175,7 @@
     <t>2008</t>
   </si>
   <si>
-    <t>裂界造物·Lv40</t>
+    <t>遗迹机兵·Lv40</t>
   </si>
   <si>
     <t>40</t>
@@ -193,7 +193,7 @@
     <t>2901</t>
   </si>
   <si>
-    <t>末日兽·演示</t>
+    <t>风蚀之核·演示</t>
   </si>
   <si>
     <t>boss</t>

</xml_diff>